<commit_message>
Deploying to gh-pages from @ jangjdaniel/jangjdaniel.github.io@5a8b8d125dc723864564cbdee53d395561f7d25c 🚀
</commit_message>
<xml_diff>
--- a/assets/america_canada_travel/trip_data.xlsx
+++ b/assets/america_canada_travel/trip_data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danie\OneDrive\Desktop\jangjdaniel.github.io\assets\travel_map\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danie\OneDrive\Desktop\jangjdaniel.github.io\assets\america_canada_travel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33568CBC-78FF-4388-B1CC-0879C217FFBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4117AC51-52F3-4D96-BA1C-CDBD979D7563}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="116">
   <si>
     <t>type</t>
   </si>
@@ -91,9 +91,6 @@
     <t>Plane</t>
   </si>
   <si>
-    <t>Graduate school visit at the University of Washington</t>
-  </si>
-  <si>
     <t>Washington</t>
   </si>
   <si>
@@ -223,9 +220,6 @@
     <t>Phoenix, AZ</t>
   </si>
   <si>
-    <t>Stuck in Layover</t>
-  </si>
-  <si>
     <t>Got stuck in Arizona because of American Airlines. Will never forgive them</t>
   </si>
   <si>
@@ -290,6 +284,90 @@
   </si>
   <si>
     <t>Amherst</t>
+  </si>
+  <si>
+    <t>Graduate school visit to the University of Washington</t>
+  </si>
+  <si>
+    <t>Senior trip with college friends</t>
+  </si>
+  <si>
+    <t>trip to see friends as a promise I made in 2025</t>
+  </si>
+  <si>
+    <t>spontaneous trip out of curiosity of south massachusetts</t>
+  </si>
+  <si>
+    <t>Fall River</t>
+  </si>
+  <si>
+    <t>Vermont</t>
+  </si>
+  <si>
+    <t>Bar Harbor, Augusta</t>
+  </si>
+  <si>
+    <t>Gorham, Hanover</t>
+  </si>
+  <si>
+    <t>Senior trip detour + visit Dartmouth</t>
+  </si>
+  <si>
+    <t>Missouri</t>
+  </si>
+  <si>
+    <t>St. Louis, Columbia, Kansas City</t>
+  </si>
+  <si>
+    <t>technically stepping foot in kansas</t>
+  </si>
+  <si>
+    <t>Kansas</t>
+  </si>
+  <si>
+    <t>Kansas City</t>
+  </si>
+  <si>
+    <t>Burlington</t>
+  </si>
+  <si>
+    <t>Road trip to canada with friends with a stop in Vermont… a farm?!</t>
+  </si>
+  <si>
+    <t>Kansas City, MO</t>
+  </si>
+  <si>
+    <t>Augusta, ME</t>
+  </si>
+  <si>
+    <t>second leg of midwest travel in 2026</t>
+  </si>
+  <si>
+    <t>Illinois</t>
+  </si>
+  <si>
+    <t>Chicago</t>
+  </si>
+  <si>
+    <t>Columbia, MO</t>
+  </si>
+  <si>
+    <t>Plane, Bus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plane  </t>
+  </si>
+  <si>
+    <t>Unwanted</t>
+  </si>
+  <si>
+    <t>Fourth New Jersey food trip</t>
+  </si>
+  <si>
+    <t>Montreal, QC</t>
+  </si>
+  <si>
+    <t>Chicago, IL</t>
   </si>
 </sst>
 </file>
@@ -330,9 +408,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -629,14 +708,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J36"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.44140625" customWidth="1"/>
     <col min="2" max="2" width="60.5546875" customWidth="1"/>
     <col min="3" max="3" width="15.33203125" customWidth="1"/>
     <col min="4" max="4" width="23.6640625" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="5" max="5" width="17" customWidth="1"/>
     <col min="7" max="7" width="21.109375" customWidth="1"/>
     <col min="9" max="9" width="18.6640625" customWidth="1"/>
     <col min="10" max="10" width="19.33203125" customWidth="1"/>
@@ -679,28 +758,28 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>106</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>107</v>
       </c>
       <c r="D2" t="s">
-        <v>13</v>
+        <v>108</v>
       </c>
       <c r="E2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2" s="1">
-        <v>46130</v>
+        <v>109</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46213</v>
       </c>
       <c r="G2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" s="1">
-        <v>46132</v>
+        <v>21</v>
+      </c>
+      <c r="H2" s="2">
+        <v>46216</v>
       </c>
       <c r="I2" t="s">
-        <v>15</v>
+        <v>111</v>
       </c>
       <c r="J2" t="s">
         <v>16</v>
@@ -708,31 +787,31 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>90</v>
       </c>
       <c r="C3" t="s">
-        <v>19</v>
+        <v>97</v>
       </c>
       <c r="D3" t="s">
-        <v>20</v>
+        <v>98</v>
       </c>
       <c r="E3" t="s">
         <v>21</v>
       </c>
-      <c r="F3" s="1">
-        <v>46096</v>
+      <c r="F3" s="2">
+        <v>46210</v>
       </c>
       <c r="G3" t="s">
-        <v>21</v>
-      </c>
-      <c r="H3" s="1">
-        <v>46098</v>
+        <v>115</v>
+      </c>
+      <c r="H3" s="2">
+        <v>46213</v>
       </c>
       <c r="I3" t="s">
-        <v>22</v>
+        <v>110</v>
       </c>
       <c r="J3" t="s">
         <v>16</v>
@@ -740,63 +819,63 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>23</v>
+        <v>99</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>100</v>
       </c>
       <c r="D4" t="s">
-        <v>25</v>
+        <v>101</v>
       </c>
       <c r="E4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" s="1">
-        <v>46078</v>
+        <v>104</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46211</v>
       </c>
       <c r="G4" t="s">
-        <v>21</v>
-      </c>
-      <c r="H4" s="1">
-        <v>46080</v>
+        <v>109</v>
+      </c>
+      <c r="H4" s="2">
+        <v>46211</v>
       </c>
       <c r="I4" t="s">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="J4" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>113</v>
       </c>
       <c r="C5" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="D5" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="E5" t="s">
         <v>21</v>
       </c>
-      <c r="F5" s="1">
-        <v>46069</v>
+      <c r="F5" s="2">
+        <v>46207</v>
       </c>
       <c r="G5" t="s">
-        <v>14</v>
-      </c>
-      <c r="H5" s="1">
-        <v>46071</v>
+        <v>21</v>
+      </c>
+      <c r="H5" s="2">
+        <v>46208</v>
       </c>
       <c r="I5" t="s">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="J5" t="s">
         <v>16</v>
@@ -804,31 +883,31 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>103</v>
       </c>
       <c r="C6" t="s">
-        <v>31</v>
+        <v>93</v>
       </c>
       <c r="D6" t="s">
-        <v>32</v>
+        <v>102</v>
       </c>
       <c r="E6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6" s="1">
-        <v>46051</v>
+        <v>114</v>
+      </c>
+      <c r="F6" s="2">
+        <v>46201</v>
       </c>
       <c r="G6" t="s">
-        <v>14</v>
-      </c>
-      <c r="H6" s="1">
-        <v>46053</v>
+        <v>21</v>
+      </c>
+      <c r="H6" s="2">
+        <v>46202</v>
       </c>
       <c r="I6" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="J6" t="s">
         <v>16</v>
@@ -839,28 +918,28 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>34</v>
+        <v>91</v>
       </c>
       <c r="C7" t="s">
-        <v>35</v>
+        <v>86</v>
       </c>
       <c r="D7" t="s">
-        <v>36</v>
+        <v>92</v>
       </c>
       <c r="E7" t="s">
         <v>21</v>
       </c>
-      <c r="F7" s="1">
-        <v>46025</v>
+      <c r="F7" s="2">
+        <v>46170</v>
       </c>
       <c r="G7" t="s">
         <v>21</v>
       </c>
-      <c r="H7" s="1">
-        <v>46025</v>
+      <c r="H7" s="2">
+        <v>46170</v>
       </c>
       <c r="I7" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="J7" t="s">
         <v>16</v>
@@ -871,28 +950,28 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>38</v>
+        <v>89</v>
       </c>
       <c r="C8" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="D8" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="E8" t="s">
-        <v>21</v>
-      </c>
-      <c r="F8" s="1">
-        <v>45884</v>
+        <v>14</v>
+      </c>
+      <c r="F8" s="2">
+        <v>46157</v>
       </c>
       <c r="G8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H8" s="1">
-        <v>45887</v>
+        <v>14</v>
+      </c>
+      <c r="H8" s="2">
+        <v>46159</v>
       </c>
       <c r="I8" t="s">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="J8" t="s">
         <v>16</v>
@@ -903,31 +982,31 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>38</v>
+        <v>96</v>
       </c>
       <c r="C9" t="s">
-        <v>41</v>
+        <v>83</v>
       </c>
       <c r="D9" t="s">
-        <v>24</v>
+        <v>95</v>
       </c>
       <c r="E9" t="s">
-        <v>42</v>
-      </c>
-      <c r="F9" s="1">
-        <v>45850</v>
+        <v>105</v>
+      </c>
+      <c r="F9" s="2">
+        <v>46159</v>
       </c>
       <c r="G9" t="s">
-        <v>42</v>
-      </c>
-      <c r="H9" s="1">
-        <v>45850</v>
+        <v>14</v>
+      </c>
+      <c r="H9" s="2">
+        <v>46159</v>
       </c>
       <c r="I9" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="J9" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
@@ -935,28 +1014,28 @@
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="C10" t="s">
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="D10" t="s">
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="E10" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="F10" s="1">
-        <v>45802</v>
+        <v>46130</v>
       </c>
       <c r="G10" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="H10" s="1">
-        <v>45803</v>
+        <v>46132</v>
       </c>
       <c r="I10" t="s">
-        <v>46</v>
+        <v>15</v>
       </c>
       <c r="J10" t="s">
         <v>16</v>
@@ -964,31 +1043,31 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="B11" t="s">
-        <v>47</v>
+        <v>18</v>
       </c>
       <c r="C11" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="D11" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="E11" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="F11" s="1">
-        <v>45583</v>
+        <v>46096</v>
       </c>
       <c r="G11" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="H11" s="1">
-        <v>45585</v>
+        <v>46098</v>
       </c>
       <c r="I11" t="s">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="J11" t="s">
         <v>16</v>
@@ -996,63 +1075,63 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="B12" t="s">
-        <v>49</v>
+        <v>88</v>
       </c>
       <c r="C12" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="D12" t="s">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="E12" t="s">
         <v>21</v>
       </c>
       <c r="F12" s="1">
-        <v>45476</v>
+        <v>46078</v>
       </c>
       <c r="G12" t="s">
-        <v>51</v>
+        <v>21</v>
       </c>
       <c r="H12" s="1">
-        <v>45476</v>
+        <v>46080</v>
       </c>
       <c r="I12" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="J12" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>52</v>
+        <v>26</v>
       </c>
       <c r="C13" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="D13" t="s">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="E13" t="s">
         <v>21</v>
       </c>
       <c r="F13" s="1">
-        <v>45438</v>
+        <v>46069</v>
       </c>
       <c r="G13" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="H13" s="1">
-        <v>45439</v>
+        <v>46071</v>
       </c>
       <c r="I13" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="J13" t="s">
         <v>16</v>
@@ -1060,31 +1139,31 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="B14" t="s">
-        <v>53</v>
+        <v>29</v>
       </c>
       <c r="C14" t="s">
-        <v>54</v>
+        <v>30</v>
       </c>
       <c r="D14" t="s">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="E14" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="F14" s="1">
-        <v>45339</v>
+        <v>46051</v>
       </c>
       <c r="G14" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="H14" s="1">
-        <v>45339</v>
+        <v>46053</v>
       </c>
       <c r="I14" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="J14" t="s">
         <v>16</v>
@@ -1095,28 +1174,28 @@
         <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="C15" t="s">
-        <v>54</v>
+        <v>34</v>
       </c>
       <c r="D15" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="E15" t="s">
         <v>21</v>
       </c>
       <c r="F15" s="1">
-        <v>45178</v>
+        <v>46025</v>
       </c>
       <c r="G15" t="s">
         <v>21</v>
       </c>
       <c r="H15" s="1">
-        <v>45178</v>
+        <v>46025</v>
       </c>
       <c r="I15" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J15" t="s">
         <v>16</v>
@@ -1127,28 +1206,28 @@
         <v>10</v>
       </c>
       <c r="B16" t="s">
-        <v>58</v>
+        <v>37</v>
       </c>
       <c r="C16" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="D16" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="E16" t="s">
         <v>21</v>
       </c>
       <c r="F16" s="1">
-        <v>45074</v>
+        <v>45884</v>
       </c>
       <c r="G16" t="s">
         <v>21</v>
       </c>
       <c r="H16" s="1">
-        <v>45075</v>
+        <v>45887</v>
       </c>
       <c r="I16" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="J16" t="s">
         <v>16</v>
@@ -1159,31 +1238,31 @@
         <v>10</v>
       </c>
       <c r="B17" t="s">
-        <v>59</v>
+        <v>37</v>
       </c>
       <c r="C17" t="s">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="D17" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="E17" t="s">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="F17" s="1">
-        <v>44883</v>
+        <v>45850</v>
       </c>
       <c r="G17" t="s">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="H17" s="1">
-        <v>44886</v>
+        <v>45850</v>
       </c>
       <c r="I17" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="J17" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
@@ -1191,60 +1270,60 @@
         <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="C18" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="D18" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="E18" t="s">
         <v>21</v>
       </c>
       <c r="F18" s="1">
-        <v>44745</v>
+        <v>45802</v>
       </c>
       <c r="G18" t="s">
         <v>21</v>
       </c>
       <c r="H18" s="1">
-        <v>44749</v>
+        <v>45803</v>
       </c>
       <c r="I18" t="s">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="J18" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="B19" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="C19" t="s">
-        <v>64</v>
+        <v>12</v>
       </c>
       <c r="D19" t="s">
-        <v>65</v>
+        <v>13</v>
       </c>
       <c r="E19" t="s">
-        <v>66</v>
+        <v>14</v>
       </c>
       <c r="F19" s="1">
-        <v>44741</v>
+        <v>45583</v>
       </c>
       <c r="G19" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="H19" s="1">
-        <v>44743</v>
+        <v>45585</v>
       </c>
       <c r="I19" t="s">
-        <v>22</v>
+        <v>47</v>
       </c>
       <c r="J19" t="s">
         <v>16</v>
@@ -1252,31 +1331,31 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>67</v>
+        <v>10</v>
       </c>
       <c r="B20" t="s">
-        <v>68</v>
+        <v>48</v>
       </c>
       <c r="C20" t="s">
-        <v>69</v>
+        <v>12</v>
       </c>
       <c r="D20" t="s">
-        <v>70</v>
+        <v>49</v>
       </c>
       <c r="E20" t="s">
         <v>21</v>
       </c>
       <c r="F20" s="1">
-        <v>44740</v>
+        <v>45476</v>
       </c>
       <c r="G20" t="s">
-        <v>71</v>
+        <v>50</v>
       </c>
       <c r="H20" s="1">
-        <v>44741</v>
+        <v>45476</v>
       </c>
       <c r="I20" t="s">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="J20" t="s">
         <v>16</v>
@@ -1284,31 +1363,31 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="B21" t="s">
-        <v>87</v>
+        <v>51</v>
       </c>
       <c r="C21" t="s">
-        <v>88</v>
+        <v>43</v>
       </c>
       <c r="D21" t="s">
-        <v>89</v>
+        <v>44</v>
       </c>
       <c r="E21" t="s">
         <v>21</v>
       </c>
       <c r="F21" s="1">
-        <v>44669</v>
+        <v>45438</v>
       </c>
       <c r="G21" t="s">
         <v>21</v>
       </c>
       <c r="H21" s="1">
-        <v>44669</v>
+        <v>45439</v>
       </c>
       <c r="I21" t="s">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="J21" t="s">
         <v>16</v>
@@ -1316,31 +1395,31 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="B22" t="s">
-        <v>79</v>
+        <v>52</v>
       </c>
       <c r="C22" t="s">
-        <v>80</v>
+        <v>53</v>
       </c>
       <c r="D22" t="s">
-        <v>81</v>
+        <v>54</v>
       </c>
       <c r="E22" t="s">
         <v>21</v>
       </c>
       <c r="F22" s="1">
-        <v>44015</v>
+        <v>45339</v>
       </c>
       <c r="G22" t="s">
         <v>21</v>
       </c>
       <c r="H22" s="1">
-        <v>44015</v>
+        <v>45339</v>
       </c>
       <c r="I22" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J22" t="s">
         <v>16</v>
@@ -1351,28 +1430,28 @@
         <v>10</v>
       </c>
       <c r="B23" t="s">
-        <v>84</v>
+        <v>55</v>
       </c>
       <c r="C23" t="s">
-        <v>85</v>
+        <v>53</v>
       </c>
       <c r="D23" t="s">
-        <v>86</v>
+        <v>56</v>
       </c>
       <c r="E23" t="s">
         <v>21</v>
       </c>
       <c r="F23" s="1">
-        <v>43709</v>
+        <v>45116</v>
       </c>
       <c r="G23" t="s">
         <v>21</v>
       </c>
       <c r="H23" s="1">
-        <v>43710</v>
+        <v>45116</v>
       </c>
       <c r="I23" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="J23" t="s">
         <v>16</v>
@@ -1383,28 +1462,28 @@
         <v>10</v>
       </c>
       <c r="B24" t="s">
-        <v>82</v>
+        <v>57</v>
       </c>
       <c r="C24" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="D24" t="s">
-        <v>83</v>
+        <v>44</v>
       </c>
       <c r="E24" t="s">
         <v>21</v>
       </c>
       <c r="F24" s="1">
-        <v>43247</v>
+        <v>45074</v>
       </c>
       <c r="G24" t="s">
         <v>21</v>
       </c>
       <c r="H24" s="1">
-        <v>43249</v>
+        <v>45075</v>
       </c>
       <c r="I24" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J24" t="s">
         <v>16</v>
@@ -1415,25 +1494,25 @@
         <v>10</v>
       </c>
       <c r="B25" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="C25" t="s">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="D25" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="E25" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="F25" s="1">
-        <v>43178</v>
+        <v>44883</v>
       </c>
       <c r="G25" t="s">
         <v>21</v>
       </c>
       <c r="H25" s="1">
-        <v>43182</v>
+        <v>44886</v>
       </c>
       <c r="I25" t="s">
         <v>15</v>
@@ -1447,60 +1526,60 @@
         <v>10</v>
       </c>
       <c r="B26" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="C26" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="D26" t="s">
-        <v>74</v>
+        <v>61</v>
       </c>
       <c r="E26" t="s">
-        <v>75</v>
+        <v>21</v>
       </c>
       <c r="F26" s="1">
-        <v>43181</v>
+        <v>44745</v>
       </c>
       <c r="G26" t="s">
-        <v>75</v>
+        <v>21</v>
       </c>
       <c r="H26" s="1">
-        <v>43181</v>
+        <v>44749</v>
       </c>
       <c r="I26" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="J26" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="B27" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="C27" t="s">
-        <v>31</v>
+        <v>63</v>
       </c>
       <c r="D27" t="s">
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="E27" t="s">
-        <v>21</v>
+        <v>65</v>
       </c>
       <c r="F27" s="1">
-        <v>43178</v>
+        <v>44741</v>
       </c>
       <c r="G27" t="s">
-        <v>75</v>
+        <v>21</v>
       </c>
       <c r="H27" s="1">
-        <v>43178</v>
+        <v>44743</v>
       </c>
       <c r="I27" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="J27" t="s">
         <v>16</v>
@@ -1508,35 +1587,291 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
+        <v>112</v>
+      </c>
+      <c r="B28" t="s">
+        <v>66</v>
+      </c>
+      <c r="C28" t="s">
+        <v>67</v>
+      </c>
+      <c r="D28" t="s">
+        <v>68</v>
+      </c>
+      <c r="E28" t="s">
+        <v>21</v>
+      </c>
+      <c r="F28" s="1">
+        <v>44740</v>
+      </c>
+      <c r="G28" t="s">
+        <v>69</v>
+      </c>
+      <c r="H28" s="1">
+        <v>44741</v>
+      </c>
+      <c r="I28" t="s">
+        <v>22</v>
+      </c>
+      <c r="J28" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>17</v>
+      </c>
+      <c r="B29" t="s">
+        <v>85</v>
+      </c>
+      <c r="C29" t="s">
+        <v>86</v>
+      </c>
+      <c r="D29" t="s">
+        <v>87</v>
+      </c>
+      <c r="E29" t="s">
+        <v>21</v>
+      </c>
+      <c r="F29" s="1">
+        <v>44669</v>
+      </c>
+      <c r="G29" t="s">
+        <v>21</v>
+      </c>
+      <c r="H29" s="1">
+        <v>44669</v>
+      </c>
+      <c r="I29" t="s">
+        <v>15</v>
+      </c>
+      <c r="J29" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>17</v>
+      </c>
+      <c r="B30" t="s">
+        <v>77</v>
+      </c>
+      <c r="C30" t="s">
         <v>78</v>
       </c>
-      <c r="B28" t="s">
-        <v>78</v>
-      </c>
-      <c r="C28" t="s">
-        <v>78</v>
-      </c>
-      <c r="D28" t="s">
-        <v>78</v>
-      </c>
-      <c r="E28" t="s">
-        <v>78</v>
-      </c>
-      <c r="F28" s="1"/>
-      <c r="G28" t="s">
-        <v>78</v>
-      </c>
-      <c r="H28" s="1"/>
-      <c r="I28" t="s">
-        <v>78</v>
-      </c>
-      <c r="J28" t="s">
-        <v>78</v>
+      <c r="D30" t="s">
+        <v>79</v>
+      </c>
+      <c r="E30" t="s">
+        <v>21</v>
+      </c>
+      <c r="F30" s="1">
+        <v>44015</v>
+      </c>
+      <c r="G30" t="s">
+        <v>21</v>
+      </c>
+      <c r="H30" s="1">
+        <v>44015</v>
+      </c>
+      <c r="I30" t="s">
+        <v>45</v>
+      </c>
+      <c r="J30" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>10</v>
+      </c>
+      <c r="B31" t="s">
+        <v>82</v>
+      </c>
+      <c r="C31" t="s">
+        <v>83</v>
+      </c>
+      <c r="D31" t="s">
+        <v>84</v>
+      </c>
+      <c r="E31" t="s">
+        <v>21</v>
+      </c>
+      <c r="F31" s="1">
+        <v>43709</v>
+      </c>
+      <c r="G31" t="s">
+        <v>21</v>
+      </c>
+      <c r="H31" s="1">
+        <v>43710</v>
+      </c>
+      <c r="I31" t="s">
+        <v>45</v>
+      </c>
+      <c r="J31" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>10</v>
+      </c>
+      <c r="B32" t="s">
+        <v>80</v>
+      </c>
+      <c r="C32" t="s">
+        <v>34</v>
+      </c>
+      <c r="D32" t="s">
+        <v>81</v>
+      </c>
+      <c r="E32" t="s">
+        <v>21</v>
+      </c>
+      <c r="F32" s="1">
+        <v>43247</v>
+      </c>
+      <c r="G32" t="s">
+        <v>21</v>
+      </c>
+      <c r="H32" s="1">
+        <v>43249</v>
+      </c>
+      <c r="I32" t="s">
+        <v>45</v>
+      </c>
+      <c r="J32" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>10</v>
+      </c>
+      <c r="B33" t="s">
+        <v>74</v>
+      </c>
+      <c r="C33" t="s">
+        <v>40</v>
+      </c>
+      <c r="D33" t="s">
+        <v>23</v>
+      </c>
+      <c r="E33" t="s">
+        <v>21</v>
+      </c>
+      <c r="F33" s="1">
+        <v>43178</v>
+      </c>
+      <c r="G33" t="s">
+        <v>21</v>
+      </c>
+      <c r="H33" s="1">
+        <v>43182</v>
+      </c>
+      <c r="I33" t="s">
+        <v>15</v>
+      </c>
+      <c r="J33" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>10</v>
+      </c>
+      <c r="B34" t="s">
+        <v>70</v>
+      </c>
+      <c r="C34" t="s">
+        <v>71</v>
+      </c>
+      <c r="D34" t="s">
+        <v>72</v>
+      </c>
+      <c r="E34" t="s">
+        <v>73</v>
+      </c>
+      <c r="F34" s="1">
+        <v>43181</v>
+      </c>
+      <c r="G34" t="s">
+        <v>73</v>
+      </c>
+      <c r="H34" s="1">
+        <v>43181</v>
+      </c>
+      <c r="I34" t="s">
+        <v>15</v>
+      </c>
+      <c r="J34" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>10</v>
+      </c>
+      <c r="B35" t="s">
+        <v>75</v>
+      </c>
+      <c r="C35" t="s">
+        <v>30</v>
+      </c>
+      <c r="D35" t="s">
+        <v>31</v>
+      </c>
+      <c r="E35" t="s">
+        <v>21</v>
+      </c>
+      <c r="F35" s="1">
+        <v>43178</v>
+      </c>
+      <c r="G35" t="s">
+        <v>73</v>
+      </c>
+      <c r="H35" s="1">
+        <v>43178</v>
+      </c>
+      <c r="I35" t="s">
+        <v>15</v>
+      </c>
+      <c r="J35" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>76</v>
+      </c>
+      <c r="B36" t="s">
+        <v>76</v>
+      </c>
+      <c r="C36" t="s">
+        <v>76</v>
+      </c>
+      <c r="D36" t="s">
+        <v>76</v>
+      </c>
+      <c r="E36" t="s">
+        <v>76</v>
+      </c>
+      <c r="F36" s="1"/>
+      <c r="G36" t="s">
+        <v>76</v>
+      </c>
+      <c r="H36" s="1"/>
+      <c r="I36" t="s">
+        <v>76</v>
+      </c>
+      <c r="J36" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J29">
-    <sortCondition descending="1" ref="H1:H29"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J38">
+    <sortCondition descending="1" ref="H1:H38"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ jangjdaniel/jangjdaniel.github.io@5121b090659ad06c0bd630396e553e38f6150a97 🚀
</commit_message>
<xml_diff>
--- a/assets/america_canada_travel/trip_data.xlsx
+++ b/assets/america_canada_travel/trip_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danie\OneDrive\Desktop\jangjdaniel.github.io\assets\america_canada_travel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4117AC51-52F3-4D96-BA1C-CDBD979D7563}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76402368-35DD-4319-B9EA-056DE2960572}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="119">
   <si>
     <t>type</t>
   </si>
@@ -368,6 +368,15 @@
   </si>
   <si>
     <t>Chicago, IL</t>
+  </si>
+  <si>
+    <t>capital_indicator</t>
+  </si>
+  <si>
+    <t>thanksgiving trip with family</t>
+  </si>
+  <si>
+    <t>Saratoga Springs</t>
   </si>
 </sst>
 </file>
@@ -708,7 +717,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J36"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.44140625" customWidth="1"/>
@@ -719,9 +728,10 @@
     <col min="7" max="7" width="21.109375" customWidth="1"/>
     <col min="9" max="9" width="18.6640625" customWidth="1"/>
     <col min="10" max="10" width="19.33203125" customWidth="1"/>
+    <col min="11" max="11" width="20.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -752,8 +762,11 @@
       <c r="J1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -784,8 +797,11 @@
       <c r="J2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -816,8 +832,11 @@
       <c r="J3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -848,8 +867,11 @@
       <c r="J4" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -880,8 +902,11 @@
       <c r="J5" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -912,8 +937,11 @@
       <c r="J6" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -944,8 +972,11 @@
       <c r="J7" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -976,8 +1007,11 @@
       <c r="J8" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -1008,8 +1042,11 @@
       <c r="J9" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -1040,8 +1077,11 @@
       <c r="J10" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -1072,8 +1112,11 @@
       <c r="J11" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>17</v>
       </c>
@@ -1104,8 +1147,11 @@
       <c r="J12" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -1136,8 +1182,11 @@
       <c r="J13" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -1168,8 +1217,11 @@
       <c r="J14" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>10</v>
       </c>
@@ -1200,8 +1252,11 @@
       <c r="J15" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K15" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>10</v>
       </c>
@@ -1232,8 +1287,11 @@
       <c r="J16" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K16" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>10</v>
       </c>
@@ -1264,8 +1322,11 @@
       <c r="J17" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K17" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>10</v>
       </c>
@@ -1296,8 +1357,11 @@
       <c r="J18" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>10</v>
       </c>
@@ -1328,8 +1392,11 @@
       <c r="J19" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K19" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>10</v>
       </c>
@@ -1360,8 +1427,11 @@
       <c r="J20" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K20" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>10</v>
       </c>
@@ -1392,8 +1462,11 @@
       <c r="J21" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K21" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>10</v>
       </c>
@@ -1424,8 +1497,11 @@
       <c r="J22" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K22" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>10</v>
       </c>
@@ -1456,8 +1532,11 @@
       <c r="J23" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K23" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>10</v>
       </c>
@@ -1488,8 +1567,11 @@
       <c r="J24" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K24" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>10</v>
       </c>
@@ -1520,8 +1602,11 @@
       <c r="J25" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K25" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>10</v>
       </c>
@@ -1552,8 +1637,11 @@
       <c r="J26" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K26" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>17</v>
       </c>
@@ -1584,8 +1672,11 @@
       <c r="J27" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K27" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>112</v>
       </c>
@@ -1616,8 +1707,11 @@
       <c r="J28" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K28" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>17</v>
       </c>
@@ -1648,8 +1742,11 @@
       <c r="J29" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K29" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>17</v>
       </c>
@@ -1680,8 +1777,11 @@
       <c r="J30" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K30" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>10</v>
       </c>
@@ -1712,8 +1812,11 @@
       <c r="J31" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K31" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>10</v>
       </c>
@@ -1744,8 +1847,11 @@
       <c r="J32" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K32" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>10</v>
       </c>
@@ -1776,8 +1882,11 @@
       <c r="J33" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K33" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>10</v>
       </c>
@@ -1808,8 +1917,11 @@
       <c r="J34" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K34" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>10</v>
       </c>
@@ -1840,8 +1952,11 @@
       <c r="J35" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K35" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>76</v>
       </c>
@@ -1867,6 +1982,41 @@
       </c>
       <c r="J36" t="s">
         <v>76</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>10</v>
+      </c>
+      <c r="B37" t="s">
+        <v>117</v>
+      </c>
+      <c r="C37" t="s">
+        <v>12</v>
+      </c>
+      <c r="D37" t="s">
+        <v>118</v>
+      </c>
+      <c r="E37" t="s">
+        <v>21</v>
+      </c>
+      <c r="F37" s="2">
+        <v>45253</v>
+      </c>
+      <c r="G37" t="s">
+        <v>14</v>
+      </c>
+      <c r="H37" s="2">
+        <v>45254</v>
+      </c>
+      <c r="I37" t="s">
+        <v>45</v>
+      </c>
+      <c r="J37" t="s">
+        <v>16</v>
+      </c>
+      <c r="K37" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
map visualizations are hard
</commit_message>
<xml_diff>
--- a/assets/america_canada_travel/trip_data.xlsx
+++ b/assets/america_canada_travel/trip_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danie\OneDrive\Desktop\jangjdaniel.github.io\assets\america_canada_travel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76402368-35DD-4319-B9EA-056DE2960572}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5BB5A8A-D132-4441-BA8A-0D24FC93DC2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1148,7 +1148,7 @@
         <v>25</v>
       </c>
       <c r="K12" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
@@ -1498,7 +1498,7 @@
         <v>16</v>
       </c>
       <c r="K22" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
@@ -1568,7 +1568,7 @@
         <v>16</v>
       </c>
       <c r="K24" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Deploying to gh-pages from @ jangjdaniel/jangjdaniel.github.io@e7def6743e16a2a7ed877ff0e815bf2db1516d95 🚀
</commit_message>
<xml_diff>
--- a/assets/america_canada_travel/trip_data.xlsx
+++ b/assets/america_canada_travel/trip_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danie\OneDrive\Desktop\jangjdaniel.github.io\assets\america_canada_travel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76402368-35DD-4319-B9EA-056DE2960572}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5BB5A8A-D132-4441-BA8A-0D24FC93DC2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1148,7 +1148,7 @@
         <v>25</v>
       </c>
       <c r="K12" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
@@ -1498,7 +1498,7 @@
         <v>16</v>
       </c>
       <c r="K22" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
@@ -1568,7 +1568,7 @@
         <v>16</v>
       </c>
       <c r="K24" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">

</xml_diff>